<commit_message>
Apply the standing table-9 no-sugar/beet/potato rule to 01.09 too
This restriction belongs to the physical table, not to whatever the
day's order text happens to spell out - it applies even when (as here)
the order text lists no exceptions for table 9 at all. Rerouted potato
mash, minestrone (has potato), sweetened porridge/drinks, cake, cookies,
and sugar packets away from S; verified no new same-day lunch/dinner
repeats were introduced.
</commit_message>
<xml_diff>
--- a/output/Гонконг 01.09.2026 (обработка).xlsx
+++ b/output/Гонконг 01.09.2026 (обработка).xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S49"/>
+  <dimension ref="A1:S56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.75" customWidth="1" min="1" max="1"/>
@@ -998,10 +998,7 @@
         <v/>
       </c>
       <c r="R6" s="15" t="n"/>
-      <c r="S6" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S6" s="15" t="n"/>
     </row>
     <row r="7" ht="37.5" customHeight="1">
       <c r="A7" s="1" t="n"/>
@@ -1032,7 +1029,10 @@
       <c r="P7" s="9" t="n"/>
       <c r="Q7" s="9" t="n"/>
       <c r="R7" s="9" t="n"/>
-      <c r="S7" s="9" t="n"/>
+      <c r="S7" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="37.5" customHeight="1">
       <c r="A8" s="13" t="n"/>
@@ -1102,187 +1102,145 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S8" s="15">
+      <c r="S8" s="15" t="n"/>
+    </row>
+    <row r="9" ht="37.5" customHeight="1">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>ЯБЛОКО ЗАПЕЧЕННОЕ</t>
+        </is>
+      </c>
+      <c r="C9" s="9">
+        <f>SUM(D9:S9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="9" t="n"/>
+      <c r="K9" s="9" t="n"/>
+      <c r="L9" s="9" t="n"/>
+      <c r="M9" s="9" t="n"/>
+      <c r="N9" s="9" t="n"/>
+      <c r="O9" s="9" t="n"/>
+      <c r="P9" s="9" t="n"/>
+      <c r="Q9" s="9" t="n"/>
+      <c r="R9" s="9" t="n"/>
+      <c r="S9" s="9">
         <f>S4</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="37.5" customHeight="1">
-      <c r="A9" s="13" t="n"/>
-      <c r="B9" s="14" t="inlineStr">
+    <row r="10" ht="37.5" customHeight="1">
+      <c r="A10" s="13" t="n"/>
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>ОМЛЕТ С ПЕРЦЕМ И ВЕТЧИНОЙ 170 ГР.</t>
         </is>
       </c>
-      <c r="C9" s="15">
-        <f>SUM(D9:S9)</f>
-        <v/>
-      </c>
-      <c r="D9" s="15" t="n"/>
-      <c r="E9" s="15">
+      <c r="C10" s="15">
+        <f>SUM(D10:S10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15">
         <f>E4</f>
         <v/>
       </c>
-      <c r="F9" s="15">
+      <c r="F10" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G9" s="15" t="n"/>
-      <c r="H9" s="15">
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I9" s="15">
+      <c r="I10" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J9" s="15">
+      <c r="J10" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K9" s="15">
+      <c r="K10" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L9" s="15">
+      <c r="L10" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M9" s="15">
+      <c r="M10" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N9" s="15">
+      <c r="N10" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O9" s="15">
+      <c r="O10" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P9" s="15">
+      <c r="P10" s="15">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q9" s="15">
+      <c r="Q10" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R9" s="15">
+      <c r="R10" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S9" s="15">
+      <c r="S10" s="15">
         <f>S4</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="37.5" customHeight="1">
-      <c r="A10" s="1" t="n"/>
-      <c r="B10" s="16" t="inlineStr">
+    <row r="11" ht="37.5" customHeight="1">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>ОМЛЕТ С ПЕРЦЕМ И ВЕТЧИНОЙ 170 ГР. БЕЗ ЛАКТОЗЫ</t>
         </is>
       </c>
-      <c r="C10" s="9">
-        <f>SUM(D10:S10)</f>
-        <v/>
-      </c>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9">
+      <c r="C11" s="9">
+        <f>SUM(D11:S11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="n"/>
-      <c r="J10" s="9" t="n"/>
-      <c r="K10" s="9" t="n"/>
-      <c r="L10" s="9" t="n"/>
-      <c r="M10" s="9" t="n"/>
-      <c r="N10" s="9" t="n"/>
-      <c r="O10" s="9" t="n"/>
-      <c r="P10" s="9" t="n"/>
-      <c r="Q10" s="9" t="n"/>
-      <c r="R10" s="9" t="n"/>
-      <c r="S10" s="9" t="n"/>
-    </row>
-    <row r="11" ht="37.5" customHeight="1">
-      <c r="A11" s="13" t="n"/>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>БУЛОЧКА ПШЕНИЧНАЯ 1 ШТ.</t>
-        </is>
-      </c>
-      <c r="C11" s="15">
-        <f>SUM(D11:S11)</f>
-        <v/>
-      </c>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G11" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H11" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I11" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J11" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K11" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L11" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M11" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N11" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O11" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P11" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q11" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R11" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S11" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="9" t="n"/>
+      <c r="M11" s="9" t="n"/>
+      <c r="N11" s="9" t="n"/>
+      <c r="O11" s="9" t="n"/>
+      <c r="P11" s="9" t="n"/>
+      <c r="Q11" s="9" t="n"/>
+      <c r="R11" s="9" t="n"/>
+      <c r="S11" s="9" t="n"/>
     </row>
     <row r="12" ht="37.5" customHeight="1">
       <c r="A12" s="13" t="n"/>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>СЛИВОЧНОЕ МАСЛО ПОРЦИОННОЕ</t>
+          <t>БУЛОЧКА ПШЕНИЧНАЯ 1 ШТ.</t>
         </is>
       </c>
       <c r="C12" s="15">
@@ -1295,7 +1253,10 @@
         <f>F4</f>
         <v/>
       </c>
-      <c r="G12" s="15" t="n"/>
+      <c r="G12" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
       <c r="H12" s="15">
         <f>H4</f>
         <v/>
@@ -1340,16 +1301,13 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S12" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S12" s="15" t="n"/>
     </row>
     <row r="13" ht="37.5" customHeight="1">
       <c r="A13" s="13" t="n"/>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>ЧАЙ 1 шт</t>
+          <t>СЛИВОЧНОЕ МАСЛО ПОРЦИОННОЕ</t>
         </is>
       </c>
       <c r="C13" s="15">
@@ -1362,10 +1320,7 @@
         <f>F4</f>
         <v/>
       </c>
-      <c r="G13" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
+      <c r="G13" s="15" t="n"/>
       <c r="H13" s="15">
         <f>H4</f>
         <v/>
@@ -1419,7 +1374,7 @@
       <c r="A14" s="13" t="n"/>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>САХАР ПОРЦИОННЫЙ</t>
+          <t>ЧАЙ 1 шт</t>
         </is>
       </c>
       <c r="C14" s="15">
@@ -1489,7 +1444,7 @@
       <c r="A15" s="13" t="n"/>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>ЛИМОН 15 гр</t>
+          <t>САХАР ПОРЦИОННЫЙ</t>
         </is>
       </c>
       <c r="C15" s="15">
@@ -1550,273 +1505,270 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S15" s="15">
+      <c r="S15" s="15" t="n"/>
+    </row>
+    <row r="16" ht="37.5" customHeight="1">
+      <c r="A16" s="13" t="n"/>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>ЛИМОН 15 гр</t>
+        </is>
+      </c>
+      <c r="C16" s="15">
+        <f>SUM(D16:S16)</f>
+        <v/>
+      </c>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G16" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H16" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I16" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J16" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K16" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L16" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M16" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N16" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O16" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P16" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q16" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R16" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S16" s="15">
         <f>S4</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="29.25" customHeight="1">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="11" t="inlineStr">
+    <row r="17" ht="29.25" customHeight="1">
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>ЗАВТРАК 2</t>
         </is>
       </c>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R16" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S16" s="12" t="inlineStr">
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R17" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S17" s="12" t="inlineStr">
         <is>
           <t>9 СТОЛ</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="37.5" customHeight="1">
-      <c r="A17" s="13" t="n"/>
-      <c r="B17" s="14" t="inlineStr">
+    <row r="18" ht="37.5" customHeight="1">
+      <c r="A18" s="13" t="n"/>
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>ФРУКТЫ СВЕЖИЕ (ЯБЛОКО)</t>
         </is>
       </c>
-      <c r="C17" s="15">
-        <f>SUM(D17:S17)</f>
-        <v/>
-      </c>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15">
+      <c r="C18" s="15">
+        <f>SUM(D18:S18)</f>
+        <v/>
+      </c>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H17" s="15">
+      <c r="H18" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I17" s="15">
+      <c r="I18" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J17" s="15">
+      <c r="J18" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K17" s="15">
+      <c r="K18" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L17" s="15">
+      <c r="L18" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M17" s="15">
+      <c r="M18" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N17" s="15">
+      <c r="N18" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O17" s="15">
+      <c r="O18" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P17" s="15">
+      <c r="P18" s="15">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q17" s="15">
+      <c r="Q18" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R17" s="15">
+      <c r="R18" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S17" s="15">
+      <c r="S18" s="15">
         <f>S4</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="37.5" customHeight="1">
-      <c r="A18" s="1" t="n"/>
-      <c r="B18" s="16" t="inlineStr">
+    <row r="19" ht="37.5" customHeight="1">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>ФРУКТЫ СВЕЖИЕ (БАНАН)</t>
         </is>
       </c>
-      <c r="C18" s="9">
-        <f>SUM(D18:S18)</f>
-        <v/>
-      </c>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9">
+      <c r="C19" s="9">
+        <f>SUM(D19:S19)</f>
+        <v/>
+      </c>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="F19" s="9">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G18" s="9" t="n"/>
-      <c r="H18" s="9" t="n"/>
-      <c r="I18" s="9" t="n"/>
-      <c r="J18" s="9" t="n"/>
-      <c r="K18" s="9" t="n"/>
-      <c r="L18" s="9" t="n"/>
-      <c r="M18" s="9" t="n"/>
-      <c r="N18" s="9" t="n"/>
-      <c r="O18" s="9" t="n"/>
-      <c r="P18" s="9" t="n"/>
-      <c r="Q18" s="9" t="n"/>
-      <c r="R18" s="9" t="n"/>
-      <c r="S18" s="9" t="n"/>
-    </row>
-    <row r="19" ht="37.5" customHeight="1">
-      <c r="A19" s="13" t="n"/>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>НАПИТОК</t>
-        </is>
-      </c>
-      <c r="C19" s="15">
-        <f>SUM(D19:S19)</f>
-        <v/>
-      </c>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G19" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H19" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I19" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J19" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K19" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L19" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M19" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N19" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O19" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P19" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q19" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R19" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S19" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="9" t="n"/>
+      <c r="I19" s="9" t="n"/>
+      <c r="J19" s="9" t="n"/>
+      <c r="K19" s="9" t="n"/>
+      <c r="L19" s="9" t="n"/>
+      <c r="M19" s="9" t="n"/>
+      <c r="N19" s="9" t="n"/>
+      <c r="O19" s="9" t="n"/>
+      <c r="P19" s="9" t="n"/>
+      <c r="Q19" s="9" t="n"/>
+      <c r="R19" s="9" t="n"/>
+      <c r="S19" s="9" t="n"/>
     </row>
     <row r="20" ht="37.5" customHeight="1">
       <c r="A20" s="13" t="n"/>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>БОУЛ ОВОЩНОЙ</t>
+          <t>НАПИТОК</t>
         </is>
       </c>
       <c r="C20" s="15">
@@ -1853,22 +1805,37 @@
         <f>L4</f>
         <v/>
       </c>
-      <c r="M20" s="15" t="n"/>
+      <c r="M20" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
       <c r="N20" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O20" s="15" t="n"/>
-      <c r="P20" s="15" t="n"/>
-      <c r="Q20" s="15" t="n"/>
-      <c r="R20" s="15" t="n"/>
+      <c r="O20" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P20" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q20" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R20" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
       <c r="S20" s="15" t="n"/>
     </row>
     <row r="21" ht="37.5" customHeight="1">
       <c r="A21" s="1" t="n"/>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>БОУЛ ОВОЩНОЙ БЕЗ КИНОА</t>
+          <t>НАПИТОК БЕЗ САХАРА</t>
         </is>
       </c>
       <c r="C21" s="9">
@@ -1884,613 +1851,553 @@
       <c r="J21" s="9" t="n"/>
       <c r="K21" s="9" t="n"/>
       <c r="L21" s="9" t="n"/>
-      <c r="M21" s="9">
-        <f>M4</f>
-        <v/>
-      </c>
+      <c r="M21" s="9" t="n"/>
       <c r="N21" s="9" t="n"/>
       <c r="O21" s="9" t="n"/>
       <c r="P21" s="9" t="n"/>
       <c r="Q21" s="9" t="n"/>
       <c r="R21" s="9" t="n"/>
-      <c r="S21" s="9" t="n"/>
-    </row>
-    <row r="22" ht="29.25" customHeight="1">
-      <c r="A22" s="10" t="n"/>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="S21" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="37.5" customHeight="1">
+      <c r="A22" s="13" t="n"/>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>БОУЛ ОВОЩНОЙ</t>
+        </is>
+      </c>
+      <c r="C22" s="15">
+        <f>SUM(D22:S22)</f>
+        <v/>
+      </c>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G22" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H22" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I22" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J22" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K22" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L22" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M22" s="15" t="n"/>
+      <c r="N22" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O22" s="15" t="n"/>
+      <c r="P22" s="15" t="n"/>
+      <c r="Q22" s="15" t="n"/>
+      <c r="R22" s="15" t="n"/>
+      <c r="S22" s="15" t="n"/>
+    </row>
+    <row r="23" ht="37.5" customHeight="1">
+      <c r="A23" s="1" t="n"/>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>БОУЛ ОВОЩНОЙ БЕЗ КИНОА</t>
+        </is>
+      </c>
+      <c r="C23" s="9">
+        <f>SUM(D23:S23)</f>
+        <v/>
+      </c>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
+      <c r="J23" s="9" t="n"/>
+      <c r="K23" s="9" t="n"/>
+      <c r="L23" s="9" t="n"/>
+      <c r="M23" s="9">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N23" s="9" t="n"/>
+      <c r="O23" s="9" t="n"/>
+      <c r="P23" s="9" t="n"/>
+      <c r="Q23" s="9" t="n"/>
+      <c r="R23" s="9" t="n"/>
+      <c r="S23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="29.25" customHeight="1">
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>ОБЕД</t>
         </is>
       </c>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R22" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S22" s="12" t="inlineStr">
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R24" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S24" s="12" t="inlineStr">
         <is>
           <t>9 СТОЛ</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="37.5" customHeight="1">
-      <c r="A23" s="13" t="n"/>
-      <c r="B23" s="14" t="inlineStr">
+    <row r="25" ht="37.5" customHeight="1">
+      <c r="A25" s="13" t="n"/>
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>САЛАТ С ТРЕСКОЙ И РИКОТТОЙ</t>
         </is>
       </c>
-      <c r="C23" s="15">
-        <f>SUM(D23:S23)</f>
-        <v/>
-      </c>
-      <c r="D23" s="15">
+      <c r="C25" s="15">
+        <f>SUM(D25:S25)</f>
+        <v/>
+      </c>
+      <c r="D25" s="15">
         <f>D4</f>
         <v/>
       </c>
-      <c r="E23" s="15">
+      <c r="E25" s="15">
         <f>E4</f>
         <v/>
       </c>
-      <c r="F23" s="15">
+      <c r="F25" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G23" s="15" t="n"/>
-      <c r="H23" s="15" t="n"/>
-      <c r="I23" s="15">
+      <c r="G25" s="15" t="n"/>
+      <c r="H25" s="15" t="n"/>
+      <c r="I25" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J23" s="15" t="n"/>
-      <c r="K23" s="15">
+      <c r="J25" s="15" t="n"/>
+      <c r="K25" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L23" s="15">
+      <c r="L25" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M23" s="15">
+      <c r="M25" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N23" s="15">
+      <c r="N25" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O23" s="15">
+      <c r="O25" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P23" s="15">
+      <c r="P25" s="15">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q23" s="15">
+      <c r="Q25" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R23" s="15">
+      <c r="R25" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S23" s="15">
+      <c r="S25" s="15">
         <f>S4</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="37.5" customHeight="1">
-      <c r="A24" s="1" t="n"/>
-      <c r="B24" s="16" t="inlineStr">
+    <row r="26" ht="37.5" customHeight="1">
+      <c r="A26" s="1" t="n"/>
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>САЛАТ С ТРЕСКОЙ И РИКОТТОЙ БЕЗ ЛАКТОЗЫ</t>
         </is>
       </c>
-      <c r="C24" s="9">
-        <f>SUM(D24:S24)</f>
-        <v/>
-      </c>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="9" t="n"/>
-      <c r="F24" s="9" t="n"/>
-      <c r="G24" s="9">
+      <c r="C26" s="9">
+        <f>SUM(D26:S26)</f>
+        <v/>
+      </c>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H24" s="9" t="n"/>
-      <c r="I24" s="9" t="n"/>
-      <c r="J24" s="9" t="n"/>
-      <c r="K24" s="9" t="n"/>
-      <c r="L24" s="9" t="n"/>
-      <c r="M24" s="9" t="n"/>
-      <c r="N24" s="9" t="n"/>
-      <c r="O24" s="9" t="n"/>
-      <c r="P24" s="9" t="n"/>
-      <c r="Q24" s="9" t="n"/>
-      <c r="R24" s="9" t="n"/>
-      <c r="S24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="37.5" customHeight="1">
-      <c r="A25" s="1" t="n"/>
-      <c r="B25" s="16" t="inlineStr">
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="9" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="9" t="n"/>
+      <c r="L26" s="9" t="n"/>
+      <c r="M26" s="9" t="n"/>
+      <c r="N26" s="9" t="n"/>
+      <c r="O26" s="9" t="n"/>
+      <c r="P26" s="9" t="n"/>
+      <c r="Q26" s="9" t="n"/>
+      <c r="R26" s="9" t="n"/>
+      <c r="S26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="37.5" customHeight="1">
+      <c r="A27" s="1" t="n"/>
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>ОВОЩНОЙ САЛАТ</t>
         </is>
       </c>
-      <c r="C25" s="9">
-        <f>SUM(D25:S25)</f>
-        <v/>
-      </c>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="9" t="n"/>
-      <c r="F25" s="9" t="n"/>
-      <c r="G25" s="9" t="n"/>
-      <c r="H25" s="9">
+      <c r="C27" s="9">
+        <f>SUM(D27:S27)</f>
+        <v/>
+      </c>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="9" t="n"/>
+      <c r="F27" s="9" t="n"/>
+      <c r="G27" s="9" t="n"/>
+      <c r="H27" s="9">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I25" s="9" t="n"/>
-      <c r="J25" s="9">
+      <c r="I27" s="9" t="n"/>
+      <c r="J27" s="9">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K25" s="9" t="n"/>
-      <c r="L25" s="9" t="n"/>
-      <c r="M25" s="9" t="n"/>
-      <c r="N25" s="9" t="n"/>
-      <c r="O25" s="9" t="n"/>
-      <c r="P25" s="9" t="n"/>
-      <c r="Q25" s="9" t="n"/>
-      <c r="R25" s="9" t="n"/>
-      <c r="S25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="37.5" customHeight="1">
-      <c r="A26" s="13" t="n"/>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="K27" s="9" t="n"/>
+      <c r="L27" s="9" t="n"/>
+      <c r="M27" s="9" t="n"/>
+      <c r="N27" s="9" t="n"/>
+      <c r="O27" s="9" t="n"/>
+      <c r="P27" s="9" t="n"/>
+      <c r="Q27" s="9" t="n"/>
+      <c r="R27" s="9" t="n"/>
+      <c r="S27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="37.5" customHeight="1">
+      <c r="A28" s="13" t="n"/>
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>СУП МИНЕСТРОНЕ</t>
         </is>
       </c>
-      <c r="C26" s="15">
-        <f>SUM(D26:S26)</f>
-        <v/>
-      </c>
-      <c r="D26" s="15">
+      <c r="C28" s="15">
+        <f>SUM(D28:S28)</f>
+        <v/>
+      </c>
+      <c r="D28" s="15">
         <f>D4</f>
         <v/>
       </c>
-      <c r="E26" s="15">
+      <c r="E28" s="15">
         <f>E4</f>
         <v/>
       </c>
-      <c r="F26" s="15">
+      <c r="F28" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G26" s="15">
+      <c r="G28" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H26" s="15">
+      <c r="H28" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I26" s="15">
+      <c r="I28" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J26" s="15">
+      <c r="J28" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K26" s="15">
+      <c r="K28" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L26" s="15">
+      <c r="L28" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M26" s="15">
+      <c r="M28" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N26" s="15">
+      <c r="N28" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O26" s="15">
+      <c r="O28" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P26" s="15">
+      <c r="P28" s="15">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q26" s="15">
+      <c r="Q28" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R26" s="15">
+      <c r="R28" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S26" s="15">
+      <c r="S28" s="15" t="n"/>
+    </row>
+    <row r="29" ht="37.5" customHeight="1">
+      <c r="A29" s="1" t="n"/>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>ТЫКВЕННЫЙ КРЕМ СУП</t>
+        </is>
+      </c>
+      <c r="C29" s="9">
+        <f>SUM(D29:S29)</f>
+        <v/>
+      </c>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="9" t="n"/>
+      <c r="I29" s="9" t="n"/>
+      <c r="J29" s="9" t="n"/>
+      <c r="K29" s="9" t="n"/>
+      <c r="L29" s="9" t="n"/>
+      <c r="M29" s="9" t="n"/>
+      <c r="N29" s="9" t="n"/>
+      <c r="O29" s="9" t="n"/>
+      <c r="P29" s="9" t="n"/>
+      <c r="Q29" s="9" t="n"/>
+      <c r="R29" s="9" t="n"/>
+      <c r="S29" s="9">
         <f>S4</f>
         <v/>
       </c>
     </row>
-    <row r="27" ht="37.5" customHeight="1">
-      <c r="A27" s="13" t="n"/>
-      <c r="B27" s="14" t="inlineStr">
+    <row r="30" ht="37.5" customHeight="1">
+      <c r="A30" s="13" t="n"/>
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>ГОВЯДИНА ДЕМИГЛЯСС</t>
         </is>
       </c>
-      <c r="C27" s="15">
-        <f>SUM(D27:S27)</f>
-        <v/>
-      </c>
-      <c r="D27" s="15">
+      <c r="C30" s="15">
+        <f>SUM(D30:S30)</f>
+        <v/>
+      </c>
+      <c r="D30" s="15">
         <f>D4</f>
         <v/>
       </c>
-      <c r="E27" s="15">
+      <c r="E30" s="15">
         <f>E4</f>
         <v/>
       </c>
-      <c r="F27" s="15">
+      <c r="F30" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G27" s="15">
+      <c r="G30" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H27" s="15">
+      <c r="H30" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I27" s="15">
+      <c r="I30" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J27" s="15">
+      <c r="J30" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K27" s="15">
+      <c r="K30" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L27" s="15">
+      <c r="L30" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M27" s="15">
+      <c r="M30" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N27" s="15">
+      <c r="N30" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O27" s="15">
+      <c r="O30" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P27" s="15">
+      <c r="P30" s="15">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q27" s="15" t="n"/>
-      <c r="R27" s="15">
+      <c r="Q30" s="15" t="n"/>
+      <c r="R30" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S27" s="15">
+      <c r="S30" s="15">
         <f>S4</f>
         <v/>
       </c>
     </row>
-    <row r="28" ht="37.5" customHeight="1">
-      <c r="A28" s="1" t="n"/>
-      <c r="B28" s="16" t="inlineStr">
+    <row r="31" ht="37.5" customHeight="1">
+      <c r="A31" s="1" t="n"/>
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>ГРУДКА КУРИНАЯ</t>
         </is>
       </c>
-      <c r="C28" s="9">
-        <f>SUM(D28:S28)</f>
-        <v/>
-      </c>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
-      <c r="F28" s="9" t="n"/>
-      <c r="G28" s="9" t="n"/>
-      <c r="H28" s="9" t="n"/>
-      <c r="I28" s="9" t="n"/>
-      <c r="J28" s="9" t="n"/>
-      <c r="K28" s="9" t="n"/>
-      <c r="L28" s="9" t="n"/>
-      <c r="M28" s="9" t="n"/>
-      <c r="N28" s="9" t="n"/>
-      <c r="O28" s="9" t="n"/>
-      <c r="P28" s="9" t="n"/>
-      <c r="Q28" s="9">
+      <c r="C31" s="9">
+        <f>SUM(D31:S31)</f>
+        <v/>
+      </c>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="9" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9" t="n"/>
+      <c r="I31" s="9" t="n"/>
+      <c r="J31" s="9" t="n"/>
+      <c r="K31" s="9" t="n"/>
+      <c r="L31" s="9" t="n"/>
+      <c r="M31" s="9" t="n"/>
+      <c r="N31" s="9" t="n"/>
+      <c r="O31" s="9" t="n"/>
+      <c r="P31" s="9" t="n"/>
+      <c r="Q31" s="9">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R28" s="9" t="n"/>
-      <c r="S28" s="9" t="n"/>
-    </row>
-    <row r="29" ht="37.5" customHeight="1">
-      <c r="A29" s="13" t="n"/>
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>КАРТОФЕЛЬНОЕ ПЮРЕ</t>
-        </is>
-      </c>
-      <c r="C29" s="15">
-        <f>SUM(D29:S29)</f>
-        <v/>
-      </c>
-      <c r="D29" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E29" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
-      <c r="F29" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G29" s="15" t="n"/>
-      <c r="H29" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I29" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J29" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K29" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L29" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M29" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N29" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O29" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P29" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q29" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R29" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S29" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="37.5" customHeight="1">
-      <c r="A30" s="1" t="n"/>
-      <c r="B30" s="16" t="inlineStr">
-        <is>
-          <t>КАРТОФЕЛЬНОЕ ПЮРЕ НА ВОДЕ</t>
-        </is>
-      </c>
-      <c r="C30" s="9">
-        <f>SUM(D30:S30)</f>
-        <v/>
-      </c>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="9" t="n"/>
-      <c r="G30" s="9">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H30" s="9" t="n"/>
-      <c r="I30" s="9" t="n"/>
-      <c r="J30" s="9" t="n"/>
-      <c r="K30" s="9" t="n"/>
-      <c r="L30" s="9" t="n"/>
-      <c r="M30" s="9" t="n"/>
-      <c r="N30" s="9" t="n"/>
-      <c r="O30" s="9" t="n"/>
-      <c r="P30" s="9" t="n"/>
-      <c r="Q30" s="9" t="n"/>
-      <c r="R30" s="9" t="n"/>
-      <c r="S30" s="9" t="n"/>
-    </row>
-    <row r="31" ht="37.5" customHeight="1">
-      <c r="A31" s="13" t="n"/>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>НАПИТОК</t>
-        </is>
-      </c>
-      <c r="C31" s="15">
-        <f>SUM(D31:S31)</f>
-        <v/>
-      </c>
-      <c r="D31" s="15" t="n"/>
-      <c r="E31" s="15" t="n"/>
-      <c r="F31" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G31" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H31" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I31" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J31" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K31" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L31" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M31" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N31" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O31" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P31" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q31" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R31" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S31" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="R31" s="9" t="n"/>
+      <c r="S31" s="9" t="n"/>
     </row>
     <row r="32" ht="37.5" customHeight="1">
       <c r="A32" s="13" t="n"/>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
+          <t>КАРТОФЕЛЬНОЕ ПЮРЕ</t>
         </is>
       </c>
       <c r="C32" s="15">
         <f>SUM(D32:S32)</f>
         <v/>
       </c>
-      <c r="D32" s="15" t="n"/>
-      <c r="E32" s="15" t="n"/>
+      <c r="D32" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E32" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
       <c r="F32" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G32" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
+      <c r="G32" s="15" t="n"/>
       <c r="H32" s="15">
         <f>H4</f>
         <v/>
@@ -2535,166 +2442,66 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S32" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="29.25" customHeight="1">
-      <c r="A33" s="10" t="n"/>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>ПОЛДНИК</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="n"/>
-      <c r="D33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R33" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S33" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
+      <c r="S32" s="15" t="n"/>
+    </row>
+    <row r="33" ht="37.5" customHeight="1">
+      <c r="A33" s="1" t="n"/>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>КАРТОФЕЛЬНОЕ ПЮРЕ НА ВОДЕ</t>
+        </is>
+      </c>
+      <c r="C33" s="9">
+        <f>SUM(D33:S33)</f>
+        <v/>
+      </c>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="9" t="n"/>
+      <c r="G33" s="9">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H33" s="9" t="n"/>
+      <c r="I33" s="9" t="n"/>
+      <c r="J33" s="9" t="n"/>
+      <c r="K33" s="9" t="n"/>
+      <c r="L33" s="9" t="n"/>
+      <c r="M33" s="9" t="n"/>
+      <c r="N33" s="9" t="n"/>
+      <c r="O33" s="9" t="n"/>
+      <c r="P33" s="9" t="n"/>
+      <c r="Q33" s="9" t="n"/>
+      <c r="R33" s="9" t="n"/>
+      <c r="S33" s="9" t="n"/>
     </row>
     <row r="34" ht="37.5" customHeight="1">
-      <c r="A34" s="13" t="n"/>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>НАПИТОК</t>
-        </is>
-      </c>
-      <c r="C34" s="15">
+      <c r="A34" s="1" t="n"/>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>СПАГЕТТИ</t>
+        </is>
+      </c>
+      <c r="C34" s="9">
         <f>SUM(D34:S34)</f>
         <v/>
       </c>
-      <c r="D34" s="15" t="n"/>
-      <c r="E34" s="15" t="n"/>
-      <c r="F34" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G34" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H34" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I34" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J34" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K34" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L34" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M34" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N34" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O34" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P34" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q34" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R34" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S34" s="15">
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n"/>
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
+      <c r="J34" s="9" t="n"/>
+      <c r="K34" s="9" t="n"/>
+      <c r="L34" s="9" t="n"/>
+      <c r="M34" s="9" t="n"/>
+      <c r="N34" s="9" t="n"/>
+      <c r="O34" s="9" t="n"/>
+      <c r="P34" s="9" t="n"/>
+      <c r="Q34" s="9" t="n"/>
+      <c r="R34" s="9" t="n"/>
+      <c r="S34" s="9">
         <f>S4</f>
         <v/>
       </c>
@@ -2703,7 +2510,7 @@
       <c r="A35" s="13" t="n"/>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">ПЕЧЕНЬЕ </t>
+          <t>НАПИТОК</t>
         </is>
       </c>
       <c r="C35" s="15">
@@ -2764,77 +2571,35 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S35" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S35" s="15" t="n"/>
     </row>
     <row r="36" ht="37.5" customHeight="1">
-      <c r="A36" s="13" t="n"/>
-      <c r="B36" s="14" t="inlineStr">
-        <is>
-          <t>ЧАЙ</t>
-        </is>
-      </c>
-      <c r="C36" s="15">
+      <c r="A36" s="1" t="n"/>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>НАПИТОК БЕЗ САХАРА</t>
+        </is>
+      </c>
+      <c r="C36" s="9">
         <f>SUM(D36:S36)</f>
         <v/>
       </c>
-      <c r="D36" s="15" t="n"/>
-      <c r="E36" s="15" t="n"/>
-      <c r="F36" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G36" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H36" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I36" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J36" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K36" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L36" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M36" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N36" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O36" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P36" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q36" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R36" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S36" s="15">
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="9" t="n"/>
+      <c r="F36" s="9" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="9" t="n"/>
+      <c r="K36" s="9" t="n"/>
+      <c r="L36" s="9" t="n"/>
+      <c r="M36" s="9" t="n"/>
+      <c r="N36" s="9" t="n"/>
+      <c r="O36" s="9" t="n"/>
+      <c r="P36" s="9" t="n"/>
+      <c r="Q36" s="9" t="n"/>
+      <c r="R36" s="9" t="n"/>
+      <c r="S36" s="9">
         <f>S4</f>
         <v/>
       </c>
@@ -2843,7 +2608,7 @@
       <c r="A37" s="13" t="n"/>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>САХАР ПОРЦИОННЫЙ</t>
+          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
         </is>
       </c>
       <c r="C37" s="15">
@@ -2913,7 +2678,7 @@
       <c r="A38" s="10" t="n"/>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>УЖИН</t>
+          <t>ПОЛДНИК</t>
         </is>
       </c>
       <c r="C38" s="10" t="n"/>
@@ -3002,26 +2767,23 @@
       <c r="A39" s="13" t="n"/>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>САЛАТ ГРЕЧЕСКИЙ</t>
+          <t>НАПИТОК</t>
         </is>
       </c>
       <c r="C39" s="15">
         <f>SUM(D39:S39)</f>
         <v/>
       </c>
-      <c r="D39" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E39" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="15" t="n"/>
       <c r="F39" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G39" s="15" t="n"/>
+      <c r="G39" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
       <c r="H39" s="15">
         <f>H4</f>
         <v/>
@@ -3066,16 +2828,13 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S39" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S39" s="15" t="n"/>
     </row>
     <row r="40" ht="37.5" customHeight="1">
       <c r="A40" s="1" t="n"/>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>САЛАТ ГРЕЧЕСКИЙ БЕЗ ФЕТЫ</t>
+          <t>НАПИТОК БЕЗ САХАРА</t>
         </is>
       </c>
       <c r="C40" s="9">
@@ -3085,10 +2844,7 @@
       <c r="D40" s="9" t="n"/>
       <c r="E40" s="9" t="n"/>
       <c r="F40" s="9" t="n"/>
-      <c r="G40" s="9">
-        <f>G4</f>
-        <v/>
-      </c>
+      <c r="G40" s="9" t="n"/>
       <c r="H40" s="9" t="n"/>
       <c r="I40" s="9" t="n"/>
       <c r="J40" s="9" t="n"/>
@@ -3100,27 +2856,24 @@
       <c r="P40" s="9" t="n"/>
       <c r="Q40" s="9" t="n"/>
       <c r="R40" s="9" t="n"/>
-      <c r="S40" s="9" t="n"/>
+      <c r="S40" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="37.5" customHeight="1">
       <c r="A41" s="13" t="n"/>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>СУДАК ТЕРИЯКИ</t>
+          <t xml:space="preserve">ПЕЧЕНЬЕ </t>
         </is>
       </c>
       <c r="C41" s="15">
         <f>SUM(D41:S41)</f>
         <v/>
       </c>
-      <c r="D41" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E41" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="15" t="n"/>
       <c r="F41" s="15">
         <f>F4</f>
         <v/>
@@ -3129,12 +2882,18 @@
         <f>G4</f>
         <v/>
       </c>
-      <c r="H41" s="15" t="n"/>
+      <c r="H41" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
       <c r="I41" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J41" s="15" t="n"/>
+      <c r="J41" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
       <c r="K41" s="15">
         <f>K4</f>
         <v/>
@@ -3167,16 +2926,13 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S41" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S41" s="15" t="n"/>
     </row>
     <row r="42" ht="37.5" customHeight="1">
       <c r="A42" s="1" t="n"/>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>ГРУДКА КУРИНАЯ</t>
+          <t>ЯБЛОКО ЗАПЕЧЕННОЕ</t>
         </is>
       </c>
       <c r="C42" s="9">
@@ -3187,15 +2943,9 @@
       <c r="E42" s="9" t="n"/>
       <c r="F42" s="9" t="n"/>
       <c r="G42" s="9" t="n"/>
-      <c r="H42" s="9">
-        <f>H4</f>
-        <v/>
-      </c>
+      <c r="H42" s="9" t="n"/>
       <c r="I42" s="9" t="n"/>
-      <c r="J42" s="9">
-        <f>J4</f>
-        <v/>
-      </c>
+      <c r="J42" s="9" t="n"/>
       <c r="K42" s="9" t="n"/>
       <c r="L42" s="9" t="n"/>
       <c r="M42" s="9" t="n"/>
@@ -3204,27 +2954,24 @@
       <c r="P42" s="9" t="n"/>
       <c r="Q42" s="9" t="n"/>
       <c r="R42" s="9" t="n"/>
-      <c r="S42" s="9" t="n"/>
+      <c r="S42" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="37.5" customHeight="1">
       <c r="A43" s="13" t="n"/>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>КУС КУС С ОВОЩАМИ</t>
+          <t>ЧАЙ</t>
         </is>
       </c>
       <c r="C43" s="15">
         <f>SUM(D43:S43)</f>
         <v/>
       </c>
-      <c r="D43" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E43" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="15" t="n"/>
       <c r="F43" s="15">
         <f>F4</f>
         <v/>
@@ -3286,7 +3033,7 @@
       <c r="A44" s="13" t="n"/>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>ЧАЙ</t>
+          <t>САХАР ПОРЦИОННЫЙ</t>
         </is>
       </c>
       <c r="C44" s="15">
@@ -3347,102 +3094,121 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S44" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="37.5" customHeight="1">
-      <c r="A45" s="13" t="n"/>
-      <c r="B45" s="14" t="inlineStr">
-        <is>
-          <t>САХАР ПОРЦИОННЫЙ</t>
-        </is>
-      </c>
-      <c r="C45" s="15">
-        <f>SUM(D45:S45)</f>
-        <v/>
-      </c>
-      <c r="D45" s="15" t="n"/>
-      <c r="E45" s="15" t="n"/>
-      <c r="F45" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G45" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H45" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I45" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J45" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K45" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L45" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M45" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N45" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O45" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P45" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q45" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R45" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S45" s="15">
-        <f>S4</f>
-        <v/>
+      <c r="S44" s="15" t="n"/>
+    </row>
+    <row r="45" ht="29.25" customHeight="1">
+      <c r="A45" s="10" t="n"/>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>УЖИН</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="n"/>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R45" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S45" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
       </c>
     </row>
     <row r="46" ht="37.5" customHeight="1">
       <c r="A46" s="13" t="n"/>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
+          <t>САЛАТ ГРЕЧЕСКИЙ</t>
         </is>
       </c>
       <c r="C46" s="15">
         <f>SUM(D46:S46)</f>
         <v/>
       </c>
-      <c r="D46" s="15" t="n"/>
-      <c r="E46" s="15" t="n"/>
+      <c r="D46" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E46" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
       <c r="F46" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G46" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
+      <c r="G46" s="15" t="n"/>
       <c r="H46" s="15">
         <f>H4</f>
         <v/>
@@ -3492,125 +3258,70 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="29.25" customHeight="1">
-      <c r="A47" s="10" t="n"/>
-      <c r="B47" s="11" t="inlineStr">
-        <is>
-          <t>2-Й УЖИН</t>
-        </is>
-      </c>
-      <c r="C47" s="10" t="n"/>
-      <c r="D47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R47" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S47" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
+    <row r="47" ht="37.5" customHeight="1">
+      <c r="A47" s="1" t="n"/>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>САЛАТ ГРЕЧЕСКИЙ БЕЗ ФЕТЫ</t>
+        </is>
+      </c>
+      <c r="C47" s="9">
+        <f>SUM(D47:S47)</f>
+        <v/>
+      </c>
+      <c r="D47" s="9" t="n"/>
+      <c r="E47" s="9" t="n"/>
+      <c r="F47" s="9" t="n"/>
+      <c r="G47" s="9">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H47" s="9" t="n"/>
+      <c r="I47" s="9" t="n"/>
+      <c r="J47" s="9" t="n"/>
+      <c r="K47" s="9" t="n"/>
+      <c r="L47" s="9" t="n"/>
+      <c r="M47" s="9" t="n"/>
+      <c r="N47" s="9" t="n"/>
+      <c r="O47" s="9" t="n"/>
+      <c r="P47" s="9" t="n"/>
+      <c r="Q47" s="9" t="n"/>
+      <c r="R47" s="9" t="n"/>
+      <c r="S47" s="9" t="n"/>
     </row>
     <row r="48" ht="37.5" customHeight="1">
       <c r="A48" s="13" t="n"/>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>КЕФИР</t>
+          <t>СУДАК ТЕРИЯКИ</t>
         </is>
       </c>
       <c r="C48" s="15">
         <f>SUM(D48:S48)</f>
         <v/>
       </c>
-      <c r="D48" s="15" t="n"/>
-      <c r="E48" s="15" t="n"/>
+      <c r="D48" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E48" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
       <c r="F48" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G48" s="15" t="n"/>
-      <c r="H48" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
+      <c r="G48" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H48" s="15" t="n"/>
       <c r="I48" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J48" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
+      <c r="J48" s="15" t="n"/>
       <c r="K48" s="15">
         <f>K4</f>
         <v/>
@@ -3652,7 +3363,7 @@
       <c r="A49" s="1" t="n"/>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>НАПИТОК</t>
+          <t>ГРУДКА КУРИНАЯ</t>
         </is>
       </c>
       <c r="C49" s="9">
@@ -3662,13 +3373,16 @@
       <c r="D49" s="9" t="n"/>
       <c r="E49" s="9" t="n"/>
       <c r="F49" s="9" t="n"/>
-      <c r="G49" s="9">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H49" s="9" t="n"/>
+      <c r="G49" s="9" t="n"/>
+      <c r="H49" s="9">
+        <f>H4</f>
+        <v/>
+      </c>
       <c r="I49" s="9" t="n"/>
-      <c r="J49" s="9" t="n"/>
+      <c r="J49" s="9">
+        <f>J4</f>
+        <v/>
+      </c>
       <c r="K49" s="9" t="n"/>
       <c r="L49" s="9" t="n"/>
       <c r="M49" s="9" t="n"/>
@@ -3679,6 +3393,476 @@
       <c r="R49" s="9" t="n"/>
       <c r="S49" s="9" t="n"/>
     </row>
+    <row r="50" ht="37.5" customHeight="1">
+      <c r="A50" s="13" t="n"/>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>КУС КУС С ОВОЩАМИ</t>
+        </is>
+      </c>
+      <c r="C50" s="15">
+        <f>SUM(D50:S50)</f>
+        <v/>
+      </c>
+      <c r="D50" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E50" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="F50" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G50" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H50" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I50" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J50" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K50" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L50" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M50" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N50" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O50" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P50" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q50" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R50" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S50" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="37.5" customHeight="1">
+      <c r="A51" s="13" t="n"/>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>ЧАЙ</t>
+        </is>
+      </c>
+      <c r="C51" s="15">
+        <f>SUM(D51:S51)</f>
+        <v/>
+      </c>
+      <c r="D51" s="15" t="n"/>
+      <c r="E51" s="15" t="n"/>
+      <c r="F51" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G51" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H51" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I51" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J51" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K51" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L51" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M51" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N51" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O51" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P51" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q51" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R51" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S51" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="37.5" customHeight="1">
+      <c r="A52" s="13" t="n"/>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>САХАР ПОРЦИОННЫЙ</t>
+        </is>
+      </c>
+      <c r="C52" s="15">
+        <f>SUM(D52:S52)</f>
+        <v/>
+      </c>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="15" t="n"/>
+      <c r="F52" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G52" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H52" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I52" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J52" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K52" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L52" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M52" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N52" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O52" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P52" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q52" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R52" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S52" s="15" t="n"/>
+    </row>
+    <row r="53" ht="37.5" customHeight="1">
+      <c r="A53" s="13" t="n"/>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
+        </is>
+      </c>
+      <c r="C53" s="15">
+        <f>SUM(D53:S53)</f>
+        <v/>
+      </c>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="15" t="n"/>
+      <c r="F53" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G53" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H53" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I53" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J53" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K53" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L53" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M53" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N53" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O53" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P53" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q53" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R53" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S53" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="29.25" customHeight="1">
+      <c r="A54" s="10" t="n"/>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>2-Й УЖИН</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="n"/>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R54" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S54" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="37.5" customHeight="1">
+      <c r="A55" s="13" t="n"/>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>КЕФИР</t>
+        </is>
+      </c>
+      <c r="C55" s="15">
+        <f>SUM(D55:S55)</f>
+        <v/>
+      </c>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="15" t="n"/>
+      <c r="F55" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G55" s="15" t="n"/>
+      <c r="H55" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I55" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J55" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K55" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L55" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M55" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N55" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O55" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P55" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q55" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R55" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S55" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="37.5" customHeight="1">
+      <c r="A56" s="1" t="n"/>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>НАПИТОК</t>
+        </is>
+      </c>
+      <c r="C56" s="9">
+        <f>SUM(D56:S56)</f>
+        <v/>
+      </c>
+      <c r="D56" s="9" t="n"/>
+      <c r="E56" s="9" t="n"/>
+      <c r="F56" s="9" t="n"/>
+      <c r="G56" s="9">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H56" s="9" t="n"/>
+      <c r="I56" s="9" t="n"/>
+      <c r="J56" s="9" t="n"/>
+      <c r="K56" s="9" t="n"/>
+      <c r="L56" s="9" t="n"/>
+      <c r="M56" s="9" t="n"/>
+      <c r="N56" s="9" t="n"/>
+      <c r="O56" s="9" t="n"/>
+      <c r="P56" s="9" t="n"/>
+      <c r="Q56" s="9" t="n"/>
+      <c r="R56" s="9" t="n"/>
+      <c r="S56" s="9" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>